<commit_message>
chore: consolida baseline do repositório
</commit_message>
<xml_diff>
--- a/02-Execucao/01-Questionario/04-Resultados_iGovTI/03-pos-comentarios-gestor/20260716-iGovTI-2026-Ajustado-Comparavel.xlsx
+++ b/02-Execucao/01-Questionario/04-Resultados_iGovTI/03-pos-comentarios-gestor/20260716-iGovTI-2026-Ajustado-Comparavel.xlsx
@@ -723,7 +723,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.1806676605496295</v>
+        <v>0.1947129041438871</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -743,7 +743,7 @@
         <v>0.051372716534058</v>
       </c>
       <c r="H5" t="n">
-        <v>0.42625</v>
+        <v>0.51125</v>
       </c>
       <c r="I5" t="n">
         <v>0.1793967191405526</v>
@@ -776,7 +776,7 @@
         <v>0.3123939907216829</v>
       </c>
       <c r="S5" t="n">
-        <v>0.309962604565201</v>
+        <v>0.3380530917537163</v>
       </c>
       <c r="T5" t="n">
         <v>0.6549125350595204</v>
@@ -987,7 +987,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.3018951793437764</v>
+        <v>0.3054830036092623</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1013,7 +1013,7 @@
         <v>0.1670031774765376</v>
       </c>
       <c r="J9" t="n">
-        <v>0.1146545354858269</v>
+        <v>0.2167636551934384</v>
       </c>
       <c r="K9" t="n">
         <v>0.15</v>
@@ -1025,7 +1025,7 @@
         <v>0.7379575407672525</v>
       </c>
       <c r="N9" t="n">
-        <v>0.1745340408288195</v>
+        <v>0.184298316440158</v>
       </c>
       <c r="O9" t="n">
         <v>0.15</v>
@@ -1034,13 +1034,13 @@
         <v>0.15</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.2600424218276572</v>
+        <v>0.2625465932028756</v>
       </c>
       <c r="R9" t="n">
-        <v>0.1643424662863211</v>
+        <v>0.1838241063081691</v>
       </c>
       <c r="S9" t="n">
-        <v>0.4132183981714049</v>
+        <v>0.4203940467023767</v>
       </c>
       <c r="T9" t="n">
         <v>0.02507602242131295</v>
@@ -1053,7 +1053,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>0.05391629137736587</v>
+        <v>0.05396013116243505</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1091,7 +1091,7 @@
         <v>0.1591957468445924</v>
       </c>
       <c r="N10" t="n">
-        <v>0.1597642756113385</v>
+        <v>0.1646464134170078</v>
       </c>
       <c r="O10" t="n">
         <v>0</v>
@@ -1100,13 +1100,13 @@
         <v>0.2375</v>
       </c>
       <c r="Q10" t="n">
-        <v>0.07538941309969968</v>
+        <v>0.0766414987873089</v>
       </c>
       <c r="R10" t="n">
-        <v>0.1422425115544903</v>
+        <v>0.1424805585847111</v>
       </c>
       <c r="S10" t="n">
-        <v>0.1078325827547317</v>
+        <v>0.1079202623248701</v>
       </c>
       <c r="T10" t="n">
         <v>0.1499999999999999</v>
@@ -2109,7 +2109,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>0.5530063887842832</v>
+        <v>0.5389611451900256</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2129,7 +2129,7 @@
         <v>0.6117987287583319</v>
       </c>
       <c r="H26" t="n">
-        <v>0.8300000000000001</v>
+        <v>0.745</v>
       </c>
       <c r="I26" t="n">
         <v>0.026970637397583</v>
@@ -2162,7 +2162,7 @@
         <v>0.5750169446062644</v>
       </c>
       <c r="S26" t="n">
-        <v>0.4942140488102346</v>
+        <v>0.4661235616217193</v>
       </c>
       <c r="T26" t="n">
         <v>0.1249239775786869</v>
@@ -2561,7 +2561,7 @@
         <v>0.000490036092609412</v>
       </c>
       <c r="T32" t="n">
-        <v>0.7684437828976594</v>
+        <v>0.999999999999999</v>
       </c>
     </row>
     <row r="33">
@@ -3231,7 +3231,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>0.6636765201862554</v>
+        <v>0.6759476251518357</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -3251,13 +3251,13 @@
         <v>0.8366613446126938</v>
       </c>
       <c r="H43" t="n">
-        <v>0.915</v>
+        <v>1</v>
       </c>
       <c r="I43" t="n">
         <v>0.0693100639045635</v>
       </c>
       <c r="J43" t="n">
-        <v>0.5733156286047514</v>
+        <v>0.5282490061751518</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
@@ -3269,7 +3269,7 @@
         <v>0.7881448157309003</v>
       </c>
       <c r="N43" t="n">
-        <v>0.6249681045705874</v>
+        <v>0.5994298960423504</v>
       </c>
       <c r="O43" t="n">
         <v>0.2666666666666667</v>
@@ -3278,13 +3278,13 @@
         <v>1</v>
       </c>
       <c r="Q43" t="n">
-        <v>0.4514475810946988</v>
+        <v>0.44489798608977</v>
       </c>
       <c r="R43" t="n">
-        <v>0.4545667831943697</v>
+        <v>0.4449333319561813</v>
       </c>
       <c r="S43" t="n">
-        <v>0.4906916957598171</v>
+        <v>0.5152339056909777</v>
       </c>
       <c r="T43" t="n">
         <v>0.4952341854122916</v>
@@ -3693,7 +3693,7 @@
         </is>
       </c>
       <c r="B50" t="n">
-        <v>0.1293393206258521</v>
+        <v>0.13599874684323</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -3701,7 +3701,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.2277777777777778</v>
+        <v>0.2666666666666667</v>
       </c>
       <c r="E50" t="n">
         <v>0.07798508700049113</v>
@@ -3710,7 +3710,7 @@
         <v>0.15</v>
       </c>
       <c r="G50" t="n">
-        <v>0.1518389316326444</v>
+        <v>0.1651577840674002</v>
       </c>
       <c r="H50" t="n">
         <v>0.1</v>
@@ -3815,7 +3815,7 @@
         <v>0.4014125113872196</v>
       </c>
       <c r="T51" t="n">
-        <v>0.167173482808753</v>
+        <v>0.138753990731265</v>
       </c>
     </row>
     <row r="52">
@@ -4155,7 +4155,7 @@
         </is>
       </c>
       <c r="B57" t="n">
-        <v>0.1715339814212096</v>
+        <v>0.1714275133717559</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -4193,7 +4193,7 @@
         <v>0.8479843631296788</v>
       </c>
       <c r="N57" t="n">
-        <v>0.3304367400103184</v>
+        <v>0.3185801196251216</v>
       </c>
       <c r="O57" t="n">
         <v>0.15</v>
@@ -4202,13 +4202,13 @@
         <v>0</v>
       </c>
       <c r="Q57" t="n">
-        <v>0.2680668064108492</v>
+        <v>0.2650260268837983</v>
       </c>
       <c r="R57" t="n">
-        <v>0.1055696233979806</v>
+        <v>0.1049915091817301</v>
       </c>
       <c r="S57" t="n">
-        <v>0.1007101503182377</v>
+        <v>0.1004972142193302</v>
       </c>
       <c r="T57" t="n">
         <v>0.02507602242131295</v>
@@ -4287,7 +4287,7 @@
         </is>
       </c>
       <c r="B59" t="n">
-        <v>0.244316116990251</v>
+        <v>0.2226286084991179</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -4307,7 +4307,7 @@
         <v>0.3741549118764972</v>
       </c>
       <c r="H59" t="n">
-        <v>0.275</v>
+        <v>0.14375</v>
       </c>
       <c r="I59" t="n">
         <v>0.008990212465861</v>
@@ -4340,7 +4340,7 @@
         <v>0.05671163793768748</v>
       </c>
       <c r="S59" t="n">
-        <v>0.1144773221040048</v>
+        <v>0.07110230512173854</v>
       </c>
       <c r="T59" t="n">
         <v>0.6547658145877073</v>
@@ -4815,33 +4815,33 @@
         </is>
       </c>
       <c r="B67" t="n">
-        <v>0.3961517396969197</v>
+        <v>0.421132769125894</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Iniciando</t>
+          <t>Intermediário</t>
         </is>
       </c>
       <c r="D67" t="n">
         <v>0</v>
       </c>
       <c r="E67" t="n">
-        <v>0.380399470228791</v>
+        <v>0.620353584076456</v>
       </c>
       <c r="F67" t="n">
         <v>0.2714285714285715</v>
       </c>
       <c r="G67" t="n">
-        <v>0.2159932093886675</v>
+        <v>0.2986228677290474</v>
       </c>
       <c r="H67" t="n">
-        <v>0.915</v>
+        <v>0.8300000000000001</v>
       </c>
       <c r="I67" t="n">
         <v>0.08206378097959272</v>
       </c>
       <c r="J67" t="n">
-        <v>0.671942617312278</v>
+        <v>0.6051789621188397</v>
       </c>
       <c r="K67" t="n">
         <v>0.4333333333333333</v>
@@ -4865,10 +4865,10 @@
         <v>0.715327241111661</v>
       </c>
       <c r="R67" t="n">
-        <v>0.6765891338180399</v>
+        <v>0.664162430689428</v>
       </c>
       <c r="S67" t="n">
-        <v>0.576310270005172</v>
+        <v>0.5436426705227406</v>
       </c>
       <c r="T67" t="n">
         <v>0.05349551449880097</v>
@@ -5673,7 +5673,7 @@
         </is>
       </c>
       <c r="B80" t="n">
-        <v>0.1178504504813622</v>
+        <v>0.1311693029161179</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -5681,7 +5681,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.2277777777777778</v>
+        <v>0.3055555555555556</v>
       </c>
       <c r="E80" t="n">
         <v>0</v>
@@ -5690,7 +5690,7 @@
         <v>0.15</v>
       </c>
       <c r="G80" t="n">
-        <v>0.124984292672021</v>
+        <v>0.1516219975415325</v>
       </c>
       <c r="H80" t="n">
         <v>0.15</v>
@@ -6993,7 +6993,7 @@
         </is>
       </c>
       <c r="B100" t="n">
-        <v>0.2807396933030166</v>
+        <v>0.2808461613524704</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -7031,7 +7031,7 @@
         <v>0.8006406805404285</v>
       </c>
       <c r="N100" t="n">
-        <v>0.2577866143857638</v>
+        <v>0.2696432347709606</v>
       </c>
       <c r="O100" t="n">
         <v>0.2666666666666667</v>
@@ -7040,13 +7040,13 @@
         <v>0.325</v>
       </c>
       <c r="Q100" t="n">
-        <v>0.5354255077284336</v>
+        <v>0.5384662872554845</v>
       </c>
       <c r="R100" t="n">
-        <v>0.2066339293497064</v>
+        <v>0.207212043565957</v>
       </c>
       <c r="S100" t="n">
-        <v>0.1391128838858607</v>
+        <v>0.1393258199847682</v>
       </c>
       <c r="T100" t="n">
         <v>0.999999999999999</v>
@@ -7323,7 +7323,7 @@
         </is>
       </c>
       <c r="B105" t="n">
-        <v>0.2778395755053683</v>
+        <v>0.2758361132448119</v>
       </c>
       <c r="C105" t="inlineStr">
         <is>
@@ -7349,7 +7349,7 @@
         <v>0.0145926440848958</v>
       </c>
       <c r="J105" t="n">
-        <v>0.5244755941505904</v>
+        <v>0.4794089717209908</v>
       </c>
       <c r="K105" t="n">
         <v>0</v>
@@ -7361,7 +7361,7 @@
         <v>0.5831730825364287</v>
       </c>
       <c r="N105" t="n">
-        <v>0.5491780097330067</v>
+        <v>0.4981015926765328</v>
       </c>
       <c r="O105" t="n">
         <v>0.2083333333333333</v>
@@ -7370,13 +7370,13 @@
         <v>0.325</v>
       </c>
       <c r="Q105" t="n">
-        <v>0.4489289614649719</v>
+        <v>0.4358297714551145</v>
       </c>
       <c r="R105" t="n">
-        <v>0.3561395733042622</v>
+        <v>0.3452609104519636</v>
       </c>
       <c r="S105" t="n">
-        <v>0.3185729436556963</v>
+        <v>0.3145660191345835</v>
       </c>
       <c r="T105" t="n">
         <v>0.6549125350595204</v>
@@ -7851,7 +7851,7 @@
         </is>
       </c>
       <c r="B113" t="n">
-        <v>0.417536073251657</v>
+        <v>0.4034908296573994</v>
       </c>
       <c r="C113" t="inlineStr">
         <is>
@@ -7871,7 +7871,7 @@
         <v>0.4690253738497205</v>
       </c>
       <c r="H113" t="n">
-        <v>0.7025</v>
+        <v>0.6174999999999999</v>
       </c>
       <c r="I113" t="n">
         <v>0.03292228035466767</v>
@@ -7904,7 +7904,7 @@
         <v>0.3365773851967953</v>
       </c>
       <c r="S113" t="n">
-        <v>0.3660467726535935</v>
+        <v>0.3379562854650782</v>
       </c>
       <c r="T113" t="n">
         <v>0</v>

</xml_diff>